<commit_message>
Agregando nuevos scripts y exe para la versión 2
</commit_message>
<xml_diff>
--- a/public/plantilla_contactos.xlsx
+++ b/public/plantilla_contactos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rolando\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rolando\Desktop\proyectos emails\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25130778-1C1F-44F1-93B7-D2F212316833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA4D3F3-2D61-47E2-90C1-C4DAAD625BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="15375" windowHeight="7785" xr2:uid="{7CB02F50-AB0E-4552-BCC4-4EAA43319AAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7CB02F50-AB0E-4552-BCC4-4EAA43319AAA}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -456,9 +456,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ABBB90A-27BC-4C90-9B4A-95699C95B56D}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="21.75" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -475,7 +478,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -492,7 +495,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>8</v>
       </c>

</xml_diff>